<commit_message>
env configuration and config
</commit_message>
<xml_diff>
--- a/weather_data.xlsx
+++ b/weather_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -810,6 +810,70 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Lisbon</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>15.51</v>
+      </c>
+      <c r="C13" t="n">
+        <v>14.92</v>
+      </c>
+      <c r="D13" t="n">
+        <v>22.21</v>
+      </c>
+      <c r="E13" t="n">
+        <v>69</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1021</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>broken clouds</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-04-13 18:07:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Lisbon</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>15.51</v>
+      </c>
+      <c r="C14" t="n">
+        <v>14.92</v>
+      </c>
+      <c r="D14" t="n">
+        <v>22.21</v>
+      </c>
+      <c r="E14" t="n">
+        <v>69</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1021</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>broken clouds</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-04-13 18:07:47</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>